<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-06 Les gouttes du seau vert
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-06.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-06.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut remplir le seau vert avec les gouttes. Pour donner de l'eau au doudou à la maison, elle reprend seau, manteau et doudou.</t>
+          <t>Le zinc tic. Un point de gouttière brille sous une goutte. Sarah veut l'eau maintenant, dans le seau vert, pour le doudou. Elle pousse trop vite : l'eau gicle, le seau reste vide. Elle refuse de forcer, reprend seau, manteau, doudou. Au jardin, le seau penche. Elle refuse de foncer, retrouve le point. L'eau paie le début.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière fait plic, plic, plic. Une goutte tombe. Elle tombe dans la cuvette. La cuvette est grise. Tu entends, Sarah ? Plic, plic. Oui. Plic, plic. Maman essuie le rebord. Le bois est froid. Les bottes de Sarah attendent. Elles sont rouges. On met les bottes ? Oui, maman. Sarah enfile les bottes. On va au jardin ? Oui. Pour l'eau. La porte s'ouvre. En ce moment, Sarah est au jardin. La terre est fraîche. Les feuilles brillent. Je m'assois près du bac. Sarah a un seau vert. Elle a un manteau rouge. Elle a son doudou beige. De l'eau pour lui. Pour le doudou ? Oui. Sarah verse l'eau. Ça fait ploc. Ploc, maman. Ploc, oui. Je t'écoute. Sarah verse encore. Ça fait ploc, ploc. Le seau est mouillé. Tes mains sont froides ? Un peu. L'eau coule un peu. La terre devient sombre. Le doudou est sur la terre. C'est l'heure. On reprend ses affaires, avant de partir. Le seau ? Oui. Tu cherches le seau. Sarah cherche le seau. Elle le prend. J'ai le seau. Bien. L'eau vient à la maison. Le manteau est sur la chaise. Le doudou est sur la terre. Une oreille est un peu mouillée.</t>
+          <t>Le zinc de la gouttière fait tic. Une goutte y tient, ronde. Sous la goutte, un point de gouttière brille. Sarah connaît ce rebord, après la pluie. Le bois du rebord est froid. Ça sent le bois mouillé. Derrière la vitre, le jardin luisant attend. Maman essuie le rebord, sans presser. Un carré de ciel pâle touche le zinc. Maman, le point brille ! Oui. Il est sur le zinc. La cuvette grise attend dessous. Plic. La goutte tombe dans la cuvette. Un seau vert dort près des bottes. Les bottes de Sarah sont rouges. Le doudou beige est sur la chaise. Un manteau rouge pend au crochet. Je veux l'eau, maintenant ! Pour lui, dans le seau ! Tu la veux vite ? Oui, maman. En ce moment, Sarah saisit le seau vert. Le plastique est froid, un peu rêche. Elle court vers le rebord. Le seau tape contre sa jambe. Je le mets sous le zinc ! Elle pousse le seau, trop vite. L'eau gicle sur le bois. Oh. Le seau reste presque vide. Une manche du manteau tombe. Le manteau rouge glisse du crochet. Le doudou beige roule vers le pot. Ça ne veut pas. Le sourire de Sarah disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Maman se baisse à sa hauteur. Tu regardes le seau ? Sarah ramasse le seau, sans crier. Je le reprends.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière fait plic, plic, plic. Une goutte tombe. Elle tombe dans la cuvette. La cuvette est grise. Tu entends, Sarah ? Plic, plic. Oui. Plic, plic. Maman essuie le rebord. Le bois est froid. Les bottes de Sarah attendent. Elles sont rouges. On met les bottes ? Oui, maman. Sarah enfile les bottes. On va au jardin ? Oui. Pour l'eau. La porte s'ouvre. En ce moment, Sarah est au jardin. La terre est fraîche. Les feuilles brillent. Je m'assois près du bac. Sarah a un seau vert. Elle a un manteau rouge. Elle a son doudou beige. De l'eau pour lui. Pour le doudou ? Oui. Sarah verse l'eau. Ça fait ploc. Ploc, maman. Ploc, oui. Je t'écoute. Sarah verse encore. Ça fait ploc, ploc. Le seau est mouillé. Tes mains sont froides ? Un peu. L'eau coule un peu. La terre devient sombre. Le doudou est sur la terre. C'est l'heure. On reprend ses affaires, avant de partir. Le seau ? Oui. Tu cherches le seau. Sarah cherche le seau. Elle le prend. J'ai le seau. Bien. L'eau vient à la maison. Le manteau est sur la chaise. Le doudou est sur la terre. Une oreille est un peu mouillée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le zinc de la gouttière fait tic. Une goutte y tient, ronde. Sous la goutte, un &lt;emphasis level="moderate"&gt;point de gouttière&lt;/emphasis&gt; brille. Sarah connaît ce rebord, après la pluie. Le bois du rebord est froid. Ça sent le bois mouillé. Derrière la vitre, le jardin luisant attend. Maman essuie le rebord, sans presser. Un carré de ciel pâle touche le zinc. Maman, le point brille ! Oui. Il est sur le zinc. La cuvette grise attend dessous. Plic. La goutte tombe dans la cuvette. Un seau vert dort près des bottes. Les bottes de Sarah sont rouges. Le doudou beige est sur la chaise. Un manteau rouge pend au crochet. Je veux l'eau, maintenant ! Pour lui, dans le seau ! Tu la veux vite ? Oui, maman. En ce moment, Sarah saisit le seau vert. Le plastique est froid, un peu rêche. Elle court vers le rebord. Le seau tape contre sa jambe. Je le mets sous le zinc ! Elle pousse le seau, trop vite. L'eau gicle sur le bois. Oh. Le seau reste presque vide. Une manche du manteau tombe. Le manteau rouge glisse du crochet. Le doudou beige roule vers le pot. Ça ne veut pas. Le sourire de Sarah disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Maman se baisse à sa hauteur. Tu regardes le seau ? Sarah ramasse le seau, sans crier. Je le reprends.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léonie joue au jardin, près de maman. La terre est fraîche. Léonie a un seau vert. Elle a un manteau rouge. Elle a son doudou beige. Léonie verse l'eau. Ça fait ploc. Maman dit : c'est l'heure. On va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires avant de partir. Léonie cherche le seau. Elle le prend. Léonie cherche le manteau. Elle le prend. Léonie cherche le doudou. Elle le prend. Ses affaires sont dans ses mains. Maman dit : merci Léonie. Elles marchent vers la maison.&lt;/slow&gt; [pause]</t>
+          <t>Le zinc de la gouttière fait tic. Une goutte y tient, ronde. Sous la goutte, un &lt;emphasis&gt;point de gouttière&lt;/emphasis&gt; brille. Sarah connaît ce rebord, après la pluie. Le bois du rebord est froid. Ça sent le bois mouillé. Derrière la vitre, le jardin luisant attend. Maman essuie le rebord, sans presser. Un carré de ciel pâle touche le zinc. Maman, le point brille ! Oui. Il est sur le zinc. La cuvette grise attend dessous. Plic. La goutte tombe dans la cuvette. Un seau vert dort près des bottes. Les bottes de Sarah sont rouges. Le doudou beige est sur la chaise. Un manteau rouge pend au crochet. Je veux l'eau, maintenant ! Pour lui, dans le seau ! Tu la veux vite ? Oui, maman. En ce moment, Sarah saisit le seau vert. Le plastique est froid, un peu rêche. Elle court vers le rebord. Le seau tape contre sa jambe. Je le mets sous le zinc ! Elle pousse le seau, trop vite. L'eau gicle sur le bois. Oh. Le seau reste presque vide. Une manche du manteau tombe. Le manteau rouge glisse du crochet. Le doudou beige roule vers le pot. Ça ne veut pas. Le sourire de Sarah disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Maman se baisse à sa hauteur. Tu regardes le seau ? Sarah ramasse le seau, sans crier. Je le reprends. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>point de gouttière</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,66 +1324,62 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_l_eau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La gouttière fait plic, plic, plic.
-narrateur|Une goutte tombe.
-narrateur|Elle tombe dans la cuvette.
-narrateur|La cuvette est grise.
-maman|Tu entends, Sarah ?
-enfant-f|Plic, plic.
+          <t>narrateur|Le zinc de la gouttière fait tic.
+narrateur|Une goutte y tient, ronde.
+narrateur|Sous la goutte, un point de gouttière brille.
+narrateur|Sarah connaît ce rebord, après la pluie.
+narrateur|Le bois du rebord est froid.
+narrateur|Ça sent le bois mouillé.
+narrateur|Derrière la vitre, le jardin luisant attend.
+narrateur|Maman essuie le rebord, sans presser.
+narrateur|Un carré de ciel pâle touche le zinc.
+enfant-f|Maman, le point brille !
 maman|Oui.
-maman|Plic, plic.
-narrateur|Maman essuie le rebord.
-narrateur|Le bois est froid.
-narrateur|Les bottes de Sarah attendent.
-narrateur|Elles sont rouges.
-maman|On met les bottes ?
+maman|Il est sur le zinc.
+narrateur|La cuvette grise attend dessous.
+narrateur|Plic.
+narrateur|La goutte tombe dans la cuvette.
+narrateur|Un seau vert dort près des bottes.
+narrateur|Les bottes de Sarah sont rouges.
+narrateur|Le doudou beige est sur la chaise.
+narrateur|Un manteau rouge pend au crochet.
+enfant-f|Je veux l'eau, maintenant !
+enfant-f|Pour lui, dans le seau !
+maman|Tu la veux vite ?
 enfant-f|Oui, maman.
-narrateur|Sarah enfile les bottes.
-maman|On va au jardin ?
-enfant-f|Oui.
-enfant-f|Pour l'eau.
-narrateur|La porte s'ouvre.
-narrateur|En ce moment, Sarah est au jardin.
-narrateur|La terre est fraîche.
-narrateur|Les feuilles brillent.
-maman|Je m'assois près du bac.
-narrateur|Sarah a un seau vert.
-narrateur|Elle a un manteau rouge.
-narrateur|Elle a son doudou beige.
-enfant-f|De l'eau pour lui.
-maman|Pour le doudou ?
-enfant-f|Oui.
-narrateur|Sarah verse l'eau.
-narrateur|Ça fait ploc.
-enfant-f|Ploc, maman.
-maman|Ploc, oui.
-maman|Je t'écoute.
-narrateur|Sarah verse encore.
-narrateur|Ça fait ploc, ploc.
-narrateur|Le seau est mouillé.
-maman|Tes mains sont froides ?
-enfant-f|Un peu.
-narrateur|L'eau coule un peu.
-narrateur|La terre devient sombre.
-narrateur|Le doudou est sur la terre.
-maman|C'est l'heure.
-maman|On reprend ses affaires, avant de partir.
-enfant-f|Le seau ?
-maman|Oui.
-maman|Tu cherches le seau.
-narrateur|Sarah cherche le seau.
-narrateur|Elle le prend.
-enfant-f|J'ai le seau.
-maman|Bien.
-maman|L'eau vient à la maison.
-narrateur|Le manteau est sur la chaise.
-narrateur|Le doudou est sur la terre.
-narrateur|Une oreille est un peu mouillée.</t>
+narrateur|En ce moment, Sarah saisit le seau vert.
+narrateur|Le plastique est froid, un peu rêche.
+narrateur|Elle court vers le rebord.
+narrateur|Le seau tape contre sa jambe.
+enfant-f|Je le mets sous le zinc !
+narrateur|Elle pousse le seau, trop vite.
+narrateur|L'eau gicle sur le bois.
+enfant-f|Oh.
+narrateur|Le seau reste presque vide.
+narrateur|Une manche du manteau tombe.
+narrateur|Le manteau rouge glisse du crochet.
+narrateur|Le doudou beige roule vers le pot.
+enfant-f|Ça ne veut pas.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, envie et inquiétude se bousculent.
+narrateur|Maman se baisse à sa hauteur.
+maman|Tu regardes le seau ?
+narrateur|Sarah ramasse le seau, sans crier.
+enfant-f|Je le reprends.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>gouttiere,goutte,seau</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1411,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Sarah ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Avant de &lt;emphasis level="moderate"&gt;partir&lt;/emphasis&gt;, que fait Sarah ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Léonie ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Avant de &lt;emphasis&gt;partir&lt;/emphasis&gt;, que fait Sarah ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1483,7 +1479,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1491,10 +1487,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1509,38 +1505,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>partir</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1549,13 +1545,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1565,7 +1561,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_reprend_avant_de_partir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1597,17 +1593,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah cherche le manteau. Elle le prend. Le manteau. Oui. Tu cherches le doudou. Sarah cherche le doudou. Elle le prend. Le doudou. Son oreille est mouillée. Un peu. Tu as repris tes affaires. Avant de partir. Oui. Ses affaires sont dans ses mains. Elles marchent vers la maison. Les bottes font poum, poum. Tu tiens tout ? Oui.</t>
+          <t>Sarah refuse de pousser plus fort. Elle pose un genou au sol. Le seau vert est froid, vide. Je le tiens. Le manteau, près du crochet ? Sarah se penche. Le manteau rouge est un peu mouillé. Elle le prend, sans tirer. Le manteau. Oui. Le doudou beige attend près du pot. Toi aussi. Elle le ramasse, une oreille mouillée. Son oreille est froide. Tu le serres ? Oui, maman. Sarah appuie le seau contre sa hanche. Le plastique fait un petit clic. On met tes bottes ? Sarah enfile ses bottes rouges. Une semelle est froide. Tu as fini tes bottes ? Oui, maman. Tu tiens tout ? Oui. Merci, Sarah. Le seau est prêt ? Oui, maman. Sarah pose la main sur le bord. Le bord est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah cherche le manteau. Elle le prend. Le manteau. Oui. Tu cherches le doudou. Sarah cherche le doudou. Elle le prend. Le doudou. Son oreille est mouillée. Un peu. Tu as repris tes affaires. Avant de partir. Oui. Ses affaires sont dans ses mains. Elles marchent vers la maison. Les bottes font poum, poum. Tu tiens tout ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah refuse de pousser plus fort. Elle pose un genou au sol. Le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; vert est froid, vide. Je le tiens. Le manteau, près du crochet ? Sarah se penche. Le manteau rouge est un peu mouillé. Elle le prend, sans tirer. Le manteau. Oui. Le doudou beige attend près du pot. Toi aussi. Elle le ramasse, une oreille mouillée. Son oreille est froide. Tu le serres ? Oui, maman. Sarah appuie le seau contre sa hanche. Le plastique fait un petit clic. On met tes bottes ? Sarah enfile ses bottes rouges. Une semelle est froide. Tu as fini tes bottes ? Oui, maman. Tu tiens tout ? Oui. Merci, Sarah. Le seau est prêt ? Oui, maman. Sarah pose la main sur le bord. Le bord est un peu rêche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léonie a cherché. Elle a repris le seau. Elle a repris le manteau. Elle a repris le doudou. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir.&lt;/slow&gt; [pause]</t>
+          <t>Sarah refuse de pousser plus fort. Elle pose un genou au sol. Le &lt;emphasis&gt;seau&lt;/emphasis&gt; vert est froid, vide. Je le tiens. Le manteau, près du crochet ? Sarah se penche. Le manteau rouge est un peu mouillé. Elle le prend, sans tirer. Le manteau. Oui. Le doudou beige attend près du pot. Toi aussi. Elle le ramasse, une oreille mouillée. Son oreille est froide. Tu le serres ? Oui, maman. Sarah appuie le seau contre sa hanche. Le plastique fait un petit clic. On met tes bottes ? Sarah enfile ses bottes rouges. Une semelle est froide. Tu as fini tes bottes ? Oui, maman. Tu tiens tout ? Oui. Merci, Sarah. Le seau est prêt ? Oui, maman. Sarah pose la main sur le bord. Le bord est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1654,18 +1650,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1688,30 +1684,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1720,10 +1716,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1732,33 +1728,50 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_reprend_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah cherche le manteau.
-narrateur|Elle le prend.
+          <t>narrateur|Sarah refuse de pousser plus fort.
+narrateur|Elle pose un genou au sol.
+narrateur|Le seau vert est froid, vide.
+enfant-f|Je le tiens.
+maman|Le manteau, près du crochet ?
+narrateur|Sarah se penche.
+narrateur|Le manteau rouge est un peu mouillé.
+narrateur|Elle le prend, sans tirer.
 enfant-f|Le manteau.
 maman|Oui.
-maman|Tu cherches le doudou.
-narrateur|Sarah cherche le doudou.
-narrateur|Elle le prend.
-enfant-f|Le doudou.
-maman|Son oreille est mouillée.
-enfant-f|Un peu.
-maman|Tu as repris tes affaires.
-enfant-f|Avant de partir.
-maman|Oui.
-narrateur|Ses affaires sont dans ses mains.
-narrateur|Elles marchent vers la maison.
-narrateur|Les bottes font poum, poum.
+narrateur|Le doudou beige attend près du pot.
+enfant-f|Toi aussi.
+narrateur|Elle le ramasse, une oreille mouillée.
+enfant-f|Son oreille est froide.
+maman|Tu le serres ?
+enfant-f|Oui, maman.
+narrateur|Sarah appuie le seau contre sa hanche.
+narrateur|Le plastique fait un petit clic.
+maman|On met tes bottes ?
+narrateur|Sarah enfile ses bottes rouges.
+narrateur|Une semelle est froide.
+maman|Tu as fini tes bottes ?
+enfant-f|Oui, maman.
 maman|Tu tiens tout ?
-enfant-f|Oui.</t>
+enfant-f|Oui.
+maman|Merci, Sarah.
+maman|Le seau est prêt ?
+enfant-f|Oui, maman.
+narrateur|Sarah pose la main sur le bord.
+narrateur|Le bord est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,doudou,bottes</t>
         </is>
       </c>
     </row>
@@ -1785,17 +1798,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah tient le seau. Le doudou est contre elle. Maman ouvre la porte. La gouttière fait encore plic. Tu poses le seau ? Sarah pose le seau. Elle pose le manteau. Merci, Sarah. On donne de l'eau au doudou ? Oui, maman. Maman prend une soucoupe. Sarah verse une goutte. Ploc. Il boit. Bravo. Tu as repris tes affaires. Les bottes s'arrêtent. La maison est calme. Tu poses les bottes ? Sarah pose les bottes. Elles sont un peu mouillées.</t>
+          <t>On ouvre la porte ? Oui. Pour l'eau du tuyau. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin luisant s'ouvre. Un tuyau de zinc pend au mur. Sarah marche près de maman. L'herbe est un peu froide. Je le vois ! Le tuyau laisse une goutte, lente. Elle tend le seau, trop vite. Le seau penche. L'eau tombe à côté, dans l'herbe. Elle part ! Sarah veut foncer, sous le tuyau. Sarah refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. L'envie et l'inquiétude se bousculent. Personne ne dit la suite. Elle lève les yeux vers le zinc. Un point de gouttière brille, dehors. Comme au rebord ! Tu le vois, toi ? Oui, sur ce tuyau. Sarah s'accroupit, lente. Elle écoute le jardin, un instant. Une goutte tic, plus loin. Elle tient le seau, sans bouger. La goutte tombe au fond. Ça fait ploc. Ploc, maman. Tu le tiens sans presser ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah tient le seau. Le doudou est contre elle. Maman ouvre la porte. La gouttière fait encore plic. Tu poses le seau ? Sarah pose le seau. Elle pose le manteau. Merci, Sarah. On donne de l'eau au doudou ? Oui, maman. Maman prend une soucoupe. Sarah verse une goutte. Ploc. Il boit. Bravo. Tu as repris tes affaires. Les bottes s'arrêtent. La maison est calme. Tu poses les bottes ? Sarah pose les bottes. Elles sont un peu mouillées.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;On ouvre la porte ? Oui. Pour l'eau du tuyau. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin luisant s'ouvre. Un tuyau de zinc pend au mur. Sarah marche près de maman. L'herbe est un peu froide. Je le vois ! Le tuyau laisse une goutte, lente. Elle tend le seau, trop vite. Le seau penche. L'eau tombe à côté, dans l'herbe. Elle part ! Sarah veut foncer, sous le tuyau. Sarah refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. L'envie et l'inquiétude se bousculent. Personne ne dit la suite. Elle lève les yeux vers le zinc. Un &lt;emphasis level="moderate"&gt;point de gouttière&lt;/emphasis&gt; brille, dehors. Comme au rebord ! Tu le vois, toi ? Oui, sur ce tuyau. Sarah s'accroupit, lente. Elle écoute le jardin, un instant. Une goutte tic, plus loin. Elle tient le seau, sans bouger. La goutte tombe au fond. Ça fait ploc. Ploc, maman. Tu le tiens sans presser ? Oui, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léonie tient le seau. Le doudou est contre elle. Maman est à côté.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;On ouvre la porte ? Oui. Pour l'eau du tuyau. Maman ouvre la porte. L'air sent la terre mouillée. Le jardin luisant s'ouvre. Un tuyau de zinc pend au mur. Sarah marche près de maman. L'herbe est un peu froide. Je le vois ! Le tuyau laisse une goutte, lente. Elle tend le seau, trop vite. Le seau penche. L'eau tombe à côté, dans l'herbe. Elle part ! Sarah veut foncer, sous le tuyau. Sarah refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. L'envie et l'inquiétude se bousculent. Personne ne dit la suite. Elle lève les yeux vers le zinc. Un &lt;emphasis&gt;point de gouttière&lt;/emphasis&gt; brille, dehors. Comme au rebord ! Tu le vois, toi ? Oui, sur ce tuyau. Sarah s'accroupit, lente. Elle écoute le jardin, un instant. Une goutte tic, plus loin. Elle tient le seau, sans bouger. La goutte tombe au fond. Ça fait ploc. Ploc, maman. Tu le tiens sans presser ? Oui, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1842,30 +1855,34 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1874,28 +1891,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>point de gouttière</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,44 +1925,67 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_le_point; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah tient le seau.
-narrateur|Le doudou est contre elle.
+          <t>maman|On ouvre la porte ?
+enfant-f|Oui.
+enfant-f|Pour l'eau du tuyau.
 narrateur|Maman ouvre la porte.
-narrateur|La gouttière fait encore plic.
-maman|Tu poses le seau ?
-narrateur|Sarah pose le seau.
-narrateur|Elle pose le manteau.
-maman|Merci, Sarah.
-maman|On donne de l'eau au doudou ?
-enfant-f|Oui, maman.
-narrateur|Maman prend une soucoupe.
-narrateur|Sarah verse une goutte.
-narrateur|Ploc.
-enfant-f|Il boit.
-maman|Bravo.
-maman|Tu as repris tes affaires.
-narrateur|Les bottes s'arrêtent.
-narrateur|La maison est calme.
-maman|Tu poses les bottes ?
-narrateur|Sarah pose les bottes.
-narrateur|Elles sont un peu mouillées.</t>
+narrateur|L'air sent la terre mouillée.
+narrateur|Le jardin luisant s'ouvre.
+narrateur|Un tuyau de zinc pend au mur.
+narrateur|Sarah marche près de maman.
+narrateur|L'herbe est un peu froide.
+enfant-f|Je le vois !
+narrateur|Le tuyau laisse une goutte, lente.
+narrateur|Elle tend le seau, trop vite.
+narrateur|Le seau penche.
+narrateur|L'eau tombe à côté, dans l'herbe.
+enfant-f|Elle part !
+narrateur|Sarah veut foncer, sous le tuyau.
+narrateur|Sarah refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|L'envie et l'inquiétude se bousculent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle lève les yeux vers le zinc.
+narrateur|Un point de gouttière brille, dehors.
+enfant-f|Comme au rebord !
+maman|Tu le vois, toi ?
+enfant-f|Oui, sur ce tuyau.
+narrateur|Sarah s'accroupit, lente.
+narrateur|Elle écoute le jardin, un instant.
+narrateur|Une goutte tic, plus loin.
+narrateur|Elle tient le seau, sans bouger.
+narrateur|La goutte tombe au fond.
+narrateur|Ça fait ploc.
+enfant-f|Ploc, maman.
+maman|Tu le tiens sans presser ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>porte,jardin,gouttiere</t>
         </is>
       </c>
     </row>
@@ -1968,17 +2012,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a de l'eau. Et toi, tu as repris tes affaires. La gouttière fait encore plic.</t>
+          <t>Sarah tient le seau, un peu plein. L'eau tremble, claire. Elle brille, maman. Tu la portes à la maison ? Oui. Elles rentrent dans la maison. La maison est tiède. Sarah pose le seau près de la cuvette. On donne de l'eau au doudou ? Oui, maman. Maman prend une soucoupe. Sarah verse une goutte. Ploc. Il boit. Le doudou beige a le museau frais. Comme sur le zinc, maman. Sur l'eau, un point de gouttière dore. Tu le vois, sur l'eau ? Oui. C'est mon seau vert. La soucoupe garde la goutte. Le point de gouttière dore, mince.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a de l'eau. Et toi, tu as repris tes affaires. La gouttière fait encore plic.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sarah tient le seau, un peu plein. L'eau tremble, claire. Elle brille, maman. Tu la portes à la maison ? Oui. Elles rentrent dans la maison. La maison est tiède. Sarah pose le seau près de la cuvette. On donne de l'eau au doudou ? Oui, maman. Maman prend une soucoupe. Sarah verse une goutte. Ploc. Il boit. Le doudou beige a le museau frais. Comme sur le zinc, maman. Sur l'eau, un &lt;emphasis level="moderate"&gt;point de gouttière&lt;/emphasis&gt; dore. Tu le vois, sur l'eau ? Oui. C'est mon seau vert. La soucoupe garde la goutte. Le point de gouttière dore, mince.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sarah tient le seau, un peu plein. L'eau tremble, claire. Elle brille, maman. Tu la portes à la maison ? Oui. Elles rentrent dans la maison. La maison est tiède. Sarah pose le seau près de la cuvette. On donne de l'eau au doudou ? Oui, maman. Maman prend une soucoupe. Sarah verse une goutte. Ploc. Il boit. Le doudou beige a le museau frais. Comme sur le zinc, maman. Sur l'eau, un &lt;emphasis&gt;point de gouttière&lt;/emphasis&gt; dore. Tu le vois, sur l'eau ? Oui. C'est mon seau vert. La soucoupe garde la goutte. Le point de gouttière dore, mince.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2025,7 +2069,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2033,10 +2077,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2045,12 +2089,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2059,17 +2103,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>point de gouttière</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2078,11 +2126,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2091,26 +2139,54 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=le_point_de_gouttiere_est_sur_l_eau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Le doudou a de l'eau.
-maman|Et toi, tu as repris tes affaires.
-narrateur|La gouttière fait encore plic.</t>
+          <t>narrateur|Sarah tient le seau, un peu plein.
+narrateur|L'eau tremble, claire.
+enfant-f|Elle brille, maman.
+maman|Tu la portes à la maison ?
+enfant-f|Oui.
+narrateur|Elles rentrent dans la maison.
+narrateur|La maison est tiède.
+narrateur|Sarah pose le seau près de la cuvette.
+maman|On donne de l'eau au doudou ?
+enfant-f|Oui, maman.
+narrateur|Maman prend une soucoupe.
+narrateur|Sarah verse une goutte.
+narrateur|Ploc.
+enfant-f|Il boit.
+narrateur|Le doudou beige a le museau frais.
+enfant-f|Comme sur le zinc, maman.
+narrateur|Sur l'eau, un point de gouttière dore.
+maman|Tu le vois, sur l'eau ?
+enfant-f|Oui.
+enfant-f|C'est mon seau vert.
+narrateur|La soucoupe garde la goutte.
+narrateur|Le point de gouttière dore, mince.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>soucoupe,eau,doudou</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2223,6 +2299,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): polish ATOM-AUT.AFF.003-06 xlsx
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-06.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-06.xlsx
@@ -2207,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2306,6 +2306,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>